<commit_message>
dados: 2026-10-12 14:51 (108 arquivos)
</commit_message>
<xml_diff>
--- a/xlsx/carteira_mensal/Ago_2026.xlsx
+++ b/xlsx/carteira_mensal/Ago_2026.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="222" uniqueCount="113">
   <si>
     <t>Acompanhamento de Carteira</t>
   </si>
@@ -174,7 +174,7 @@
     <t>Mirza Castelo Branco de Luca</t>
   </si>
   <si>
-    <t>Indicação de Amigo</t>
+    <t>Indicação de outros clientes</t>
   </si>
   <si>
     <t>04/08/26</t>
@@ -273,9 +273,6 @@
     <t>ADRIANA REGO BARROS MAGALHÃES</t>
   </si>
   <si>
-    <t>Cliente de porta</t>
-  </si>
-  <si>
     <t>Victor Costa</t>
   </si>
   <si>
@@ -303,10 +300,16 @@
     <t>Alexandre Gleyson Araujo da Silva</t>
   </si>
   <si>
+    <t>31/08/26</t>
+  </si>
+  <si>
+    <t>Márcia Elias Abucham</t>
+  </si>
+  <si>
     <t>Quantidade de Projetos</t>
   </si>
   <si>
-    <t>19</t>
+    <t>20</t>
   </si>
   <si>
     <t>Quantidade de Orçamentos</t>
@@ -315,28 +318,28 @@
     <t>Pontuação Total</t>
   </si>
   <si>
-    <t>1.92</t>
+    <t>1.93</t>
   </si>
   <si>
     <t>Valor Total Bruto</t>
   </si>
   <si>
-    <t>714.535,53</t>
-  </si>
-  <si>
-    <t>578.179,00</t>
+    <t>711.502,66</t>
+  </si>
+  <si>
+    <t>578.479,00</t>
   </si>
   <si>
     <t>Valor Total Líquido</t>
   </si>
   <si>
-    <t>466.631,53</t>
+    <t>466.931,53</t>
   </si>
   <si>
     <t>Total Líquido sem o Per</t>
   </si>
   <si>
-    <t>461.277,50</t>
+    <t>461.577,50</t>
   </si>
   <si>
     <t>Total Diferença Financeira</t>
@@ -348,7 +351,7 @@
     <t>Total Adicional dos Ambientes</t>
   </si>
   <si>
-    <t>28.123,97</t>
+    <t>28.303,97</t>
   </si>
 </sst>
 </file>
@@ -417,7 +420,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A2:O60"/>
+  <dimension ref="A2:O61"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="53.22265625" customWidth="true" bestFit="true"/>
@@ -1330,7 +1333,7 @@
         <v>85</v>
       </c>
       <c r="B45" t="s">
-        <v>86</v>
+        <v>60</v>
       </c>
       <c r="C45" t="n">
         <v>961.0</v>
@@ -1339,16 +1342,16 @@
         <v>81</v>
       </c>
       <c r="E45" t="s">
+        <v>86</v>
+      </c>
+      <c r="F45" t="n">
+        <v>2.0</v>
+      </c>
+      <c r="G45" t="s">
         <v>87</v>
       </c>
-      <c r="F45" t="n">
-        <v>1.0</v>
-      </c>
-      <c r="G45" t="s">
+      <c r="H45" t="s">
         <v>88</v>
-      </c>
-      <c r="H45" t="s">
-        <v>89</v>
       </c>
       <c r="I45" t="n">
         <v>24990.0</v>
@@ -1369,12 +1372,12 @@
         <v>96101.0</v>
       </c>
       <c r="O45" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B46" t="s">
         <v>76</v>
@@ -1383,7 +1386,7 @@
         <v>968.0</v>
       </c>
       <c r="D46" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="E46" t="s">
         <v>49</v>
@@ -1395,7 +1398,7 @@
         <v>50</v>
       </c>
       <c r="H46" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="I46" t="n">
         <v>281.69</v>
@@ -1416,12 +1419,12 @@
         <v>96801.0</v>
       </c>
       <c r="O46" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B47" t="s">
         <v>60</v>
@@ -1430,7 +1433,7 @@
         <v>973.0</v>
       </c>
       <c r="D47" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="E47" t="s">
         <v>61</v>
@@ -1442,7 +1445,7 @@
         <v>50</v>
       </c>
       <c r="H47" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="I47" t="n">
         <v>915.0</v>
@@ -1463,15 +1466,15 @@
         <v>97301.0</v>
       </c>
       <c r="O47" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B48" t="s">
-        <v>86</v>
+        <v>60</v>
       </c>
       <c r="C48" t="n">
         <v>976.0</v>
@@ -1480,13 +1483,13 @@
         <v>74</v>
       </c>
       <c r="E48" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="F48" t="n">
         <v>1.0</v>
       </c>
       <c r="G48" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="H48" t="s">
         <v>82</v>
@@ -1515,7 +1518,7 @@
     </row>
     <row r="49">
       <c r="A49" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B49" t="s">
         <v>72</v>
@@ -1536,7 +1539,7 @@
         <v>50</v>
       </c>
       <c r="H49" t="s">
-        <v>82</v>
+        <v>95</v>
       </c>
       <c r="I49" t="n">
         <v>63824.33</v>
@@ -1551,7 +1554,7 @@
         <v>52491.27</v>
       </c>
       <c r="M49" t="n">
-        <v>1.96</v>
+        <v>2.05</v>
       </c>
       <c r="N49" t="n">
         <v>97401.0</v>
@@ -1560,20 +1563,59 @@
         <v>82</v>
       </c>
     </row>
-    <row r="52">
-      <c r="A52" s="2" t="s">
+    <row r="50">
+      <c r="A50" t="s">
         <v>96</v>
       </c>
-      <c r="B52" s="3" t="s">
-        <v>97</v>
+      <c r="B50" t="s">
+        <v>47</v>
+      </c>
+      <c r="C50" t="n">
+        <v>979.0</v>
+      </c>
+      <c r="D50" t="s">
+        <v>95</v>
+      </c>
+      <c r="E50" t="s">
+        <v>67</v>
+      </c>
+      <c r="F50" t="n">
+        <v>5.0</v>
+      </c>
+      <c r="G50" t="s">
+        <v>50</v>
+      </c>
+      <c r="H50" t="s">
+        <v>95</v>
+      </c>
+      <c r="I50" t="n">
+        <v>300.0</v>
+      </c>
+      <c r="J50" t="n">
+        <v>0.0</v>
+      </c>
+      <c r="K50" t="n">
+        <v>300.0</v>
+      </c>
+      <c r="L50" t="n">
+        <v>300.0</v>
+      </c>
+      <c r="M50" t="n">
+        <v>2.42</v>
+      </c>
+      <c r="N50" t="n">
+        <v>97901.0</v>
+      </c>
+      <c r="O50" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="B53" s="3" t="s">
         <v>98</v>
-      </c>
-      <c r="B53" s="3" t="s">
-        <v>97</v>
       </c>
     </row>
     <row r="54">
@@ -1581,20 +1623,20 @@
         <v>99</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="B55" s="3" t="s">
         <v>101</v>
-      </c>
-      <c r="B55" s="3" t="s">
-        <v>102</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="s">
-        <v>17</v>
+        <v>102</v>
       </c>
       <c r="B56" s="3" t="s">
         <v>103</v>
@@ -1602,34 +1644,42 @@
     </row>
     <row r="57">
       <c r="A57" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B57" s="3" t="s">
         <v>104</v>
-      </c>
-      <c r="B57" s="3" t="s">
-        <v>105</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="B58" s="3" t="s">
         <v>106</v>
-      </c>
-      <c r="B58" s="3" t="s">
-        <v>107</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="B59" s="3" t="s">
         <v>108</v>
-      </c>
-      <c r="B59" s="3" t="s">
-        <v>109</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="B60" s="3" t="s">
         <v>110</v>
       </c>
-      <c r="B60" s="3" t="s">
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="s">
         <v>111</v>
+      </c>
+      <c r="B61" s="3" t="s">
+        <v>112</v>
       </c>
     </row>
   </sheetData>

</xml_diff>